<commit_message>
Cockpit : retirer les 6 sparklines redondantes, garder le seul graphe utile
Critique juste : 6 courbes montant toutes pareil = zéro information (redondant
avec le YoY). Retrait des 6 mini-graphes. À la place :
- YoY coloré par SENS (vert = bon sens, ochre = défavorable) -> l'oeil tombe
  direct sur le CAC, seul KPI qui monte dans le mauvais sens ("à surveiller").
- UN seul graphe conservé : la tension (dépenses +21% décrochent au-dessus de
  l'activité +12%) — la seule visualisation qui porte un message (une divergence).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/COCKPIT_ATTERRISSAGE.xlsx
+++ b/eduservices/tagetik/COCKPIT_ATTERRISSAGE.xlsx
@@ -17,13 +17,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0.00,,&quot; M€&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.0&quot; pt&quot;"/>
-    <numFmt numFmtId="168" formatCode="#,##0&quot; €&quot;"/>
-    <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="&quot;▲ &quot;0.0%"/>
+    <numFmt numFmtId="168" formatCode="&quot;▲ &quot;0.0&quot; pt&quot;"/>
+    <numFmt numFmtId="169" formatCode="#,##0&quot; €&quot;"/>
+    <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -103,9 +104,15 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000A5A48"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <i val="1"/>
-      <color rgb="00152230"/>
-      <sz val="9"/>
+      <color rgb="000A5A48"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -122,25 +129,20 @@
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00B3641C"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00152230"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
       <i val="1"/>
       <color rgb="00B3641C"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="000A5A48"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00152230"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -178,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -206,37 +208,39 @@
     <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -334,499 +338,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Chiffre d'affaires (€)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$7:$D$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$9:$D$9</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>EBITDA (€)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$7:$D$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$10:$D$10</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Marge EBITDA %</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$7:$D$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$11:$D$11</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Leads</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$7:$D$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$13:$D$13</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Inscrits</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$7:$D$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$14:$D$14</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>CAC (€/inscrit)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <numRef>
-              <f>'Cockpit'!$B$7:$D$7</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Cockpit'!$B$15:$D$15</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="1"/>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Activité vs Dépenses (base 100)</a:t>
+              <a:t>Dépenses d'acquisition (+21%) décrochent au-dessus de l'activité (+12%)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -938,12 +450,12 @@
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>6</col>
+      <col>7</col>
       <colOff>0</colOff>
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="2304000" cy="827999"/>
+    <ext cx="5400000" cy="2880000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -953,138 +465,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>12</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2304000" cy="827999"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>18</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2304000" cy="827999"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="3" name="Chart 3"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>24</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2304000" cy="827999"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="4" name="Chart 4"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>30</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2304000" cy="827999"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="5" name="Chart 5"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId5"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>6</col>
-      <colOff>0</colOff>
-      <row>36</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2304000" cy="827999"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="6" name="Chart 6"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId6"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>13</col>
-      <colOff>0</colOff>
-      <row>17</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="4320000" cy="2340000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="7" name="Chart 7"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId7"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1389,7 +769,8 @@
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1503,6 +884,11 @@
         <f>D9/C9-1</f>
         <v/>
       </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>bon sens</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -1526,6 +912,11 @@
         <f>D10/C10-1</f>
         <v/>
       </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>bon sens</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -1533,21 +924,26 @@
           <t>Marge EBITDA %</t>
         </is>
       </c>
-      <c r="B11" s="14">
+      <c r="B11" s="15">
         <f>Données!C5/Données!B5</f>
         <v/>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="15">
         <f>Données!C6/Données!B6</f>
         <v/>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="15">
         <f>Données!C7/Données!B7</f>
         <v/>
       </c>
-      <c r="E11" s="15">
+      <c r="E11" s="16">
         <f>D11-C11</f>
         <v/>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>bon sens</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -1567,15 +963,15 @@
           <t>Leads</t>
         </is>
       </c>
-      <c r="B13" s="16">
+      <c r="B13" s="17">
         <f>Données!D5</f>
         <v/>
       </c>
-      <c r="C13" s="16">
+      <c r="C13" s="17">
         <f>Données!D6</f>
         <v/>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="17">
         <f>Données!D7</f>
         <v/>
       </c>
@@ -1583,6 +979,11 @@
         <f>D13/C13-1</f>
         <v/>
       </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>bon sens</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -1590,15 +991,15 @@
           <t>Inscrits</t>
         </is>
       </c>
-      <c r="B14" s="16">
+      <c r="B14" s="17">
         <f>Données!E5</f>
         <v/>
       </c>
-      <c r="C14" s="16">
+      <c r="C14" s="17">
         <f>Données!E6</f>
         <v/>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="17">
         <f>Données!E7</f>
         <v/>
       </c>
@@ -1606,102 +1007,112 @@
         <f>D14/C14-1</f>
         <v/>
       </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>bon sens</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>CAC (€/inscrit)</t>
         </is>
       </c>
-      <c r="B15" s="18">
+      <c r="B15" s="19">
         <f>Données!F5/Données!E5</f>
         <v/>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="19">
         <f>Données!F6/Données!E6</f>
         <v/>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="19">
         <f>Données!F7/Données!E7</f>
         <v/>
       </c>
-      <c r="E15" s="19">
+      <c r="E15" s="20">
         <f>D15/C15-1</f>
         <v/>
       </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>à surveiller</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>CAC = seul KPI en tension : le coût d'acquisition monte plus vite que le volume. C'est ce qu'on ira traiter dans le budget 2027.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>TENSION — base 100 en 2024 : activité (CA) vs dépenses d'acquisition</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t>Année</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="24" t="n">
         <v>2024</v>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="24" t="n">
         <v>2025</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="24" t="n">
         <v>2026</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="24" t="inlineStr">
+      <c r="A20" s="25" t="inlineStr">
         <is>
           <t>Activité (CA)</t>
         </is>
       </c>
-      <c r="B20" s="25">
+      <c r="B20" s="26">
         <f>Données!B5/Données!B5*100</f>
         <v/>
       </c>
-      <c r="C20" s="25">
+      <c r="C20" s="26">
         <f>Données!B6/Données!B5*100</f>
         <v/>
       </c>
-      <c r="D20" s="25">
+      <c r="D20" s="26">
         <f>Données!B7/Données!B5*100</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="24" t="inlineStr">
+      <c r="A21" s="25" t="inlineStr">
         <is>
           <t>Dépenses acq.</t>
         </is>
       </c>
-      <c r="B21" s="25">
+      <c r="B21" s="26">
         <f>Données!F5/Données!F5*100</f>
         <v/>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="26">
         <f>Données!F6/Données!F5*100</f>
         <v/>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="26">
         <f>Données!F7/Données!F5*100</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t>Message : commercial ET financier sur un écran. On progresse (CA/EBITDA), mais le CAC se dégrade -&gt; le budget 2027 doit répondre à ça.</t>
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>LE graphe qui compte : l'écart entre les 2 courbes = la dégradation du CAC. C'est ce que le budget 2027 doit corriger.</t>
         </is>
       </c>
     </row>
@@ -1729,14 +1140,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="27" t="inlineStr">
+      <c r="A1" s="28" t="inlineStr">
         <is>
           <t>DONNÉES — agrégats annuels groupe (source : compta produits + socle CRM)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="29" t="inlineStr">
         <is>
           <t>2024-2025 réalisé · 2026 atterrissage. Bleu = donnée.</t>
         </is>
@@ -1775,68 +1186,68 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>2024</t>
         </is>
       </c>
-      <c r="B5" s="29" t="n">
+      <c r="B5" s="31" t="n">
         <v>20064725</v>
       </c>
-      <c r="C5" s="29" t="n">
+      <c r="C5" s="31" t="n">
         <v>2648550</v>
       </c>
-      <c r="D5" s="30" t="n">
+      <c r="D5" s="32" t="n">
         <v>15305</v>
       </c>
-      <c r="E5" s="30" t="n">
+      <c r="E5" s="32" t="n">
         <v>1092</v>
       </c>
-      <c r="F5" s="29" t="n">
+      <c r="F5" s="31" t="n">
         <v>358819</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>2025</t>
         </is>
       </c>
-      <c r="B6" s="29" t="n">
+      <c r="B6" s="31" t="n">
         <v>21268606</v>
       </c>
-      <c r="C6" s="29" t="n">
+      <c r="C6" s="31" t="n">
         <v>2977604</v>
       </c>
-      <c r="D6" s="30" t="n">
+      <c r="D6" s="32" t="n">
         <v>16226</v>
       </c>
-      <c r="E6" s="30" t="n">
+      <c r="E6" s="32" t="n">
         <v>1159</v>
       </c>
-      <c r="F6" s="29" t="n">
+      <c r="F6" s="31" t="n">
         <v>394702</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="B7" s="29" t="n">
+      <c r="B7" s="31" t="n">
         <v>22544725</v>
       </c>
-      <c r="C7" s="29" t="n">
+      <c r="C7" s="31" t="n">
         <v>3291530</v>
       </c>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="32" t="n">
         <v>17197</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="32" t="n">
         <v>1229</v>
       </c>
-      <c r="F7" s="29" t="n">
+      <c r="F7" s="31" t="n">
         <v>434174</v>
       </c>
     </row>

</xml_diff>